<commit_message>
Split volume_bands price columns by billing cadence
</commit_message>
<xml_diff>
--- a/project-management-pricing-2026-10.xlsx
+++ b/project-management-pricing-2026-10.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1002" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1003" uniqueCount="265">
   <si>
     <t xml:space="preserve">Project management software pricing, October 2026</t>
   </si>
@@ -592,10 +592,13 @@
     <t xml:space="preserve">Seats</t>
   </si>
   <si>
-    <t xml:space="preserve">Price per seat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Annual per user</t>
+    <t xml:space="preserve">Per seat, monthly rate on annual billing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per seat, monthly rate on monthly billing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per seat per year on annual billing</t>
   </si>
   <si>
     <t xml:space="preserve">pricing page seat slider</t>
@@ -1872,11 +1875,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="74711949"/>
-        <c:axId val="5992874"/>
+        <c:axId val="43801790"/>
+        <c:axId val="7178350"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="74711949"/>
+        <c:axId val="43801790"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1942,7 +1945,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="5992874"/>
+        <c:crossAx val="7178350"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1950,7 +1953,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="5992874"/>
+        <c:axId val="7178350"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2026,7 +2029,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="74711949"/>
+        <c:crossAx val="43801790"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2425,7 +2428,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2433,17 +2436,17 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2451,22 +2454,22 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2474,22 +2477,22 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2497,7 +2500,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="23" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
   </sheetData>
@@ -11354,15 +11357,14 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="11"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11375,7 +11377,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
         <v>39</v>
       </c>
@@ -11392,9 +11394,12 @@
         <v>188</v>
       </c>
       <c r="F4" s="14" t="s">
+        <v>189</v>
+      </c>
+      <c r="G4" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="G4" s="14" t="s">
+      <c r="H4" s="14" t="s">
         <v>56</v>
       </c>
     </row>
@@ -11411,13 +11416,14 @@
       <c r="D5" s="15" t="n">
         <v>17.5</v>
       </c>
-      <c r="E5" s="15" t="n">
+      <c r="E5" s="15"/>
+      <c r="F5" s="15" t="n">
         <v>210</v>
       </c>
-      <c r="F5" s="8" t="s">
-        <v>189</v>
-      </c>
       <c r="G5" s="8" t="s">
+        <v>190</v>
+      </c>
+      <c r="H5" s="8" t="s">
         <v>65</v>
       </c>
     </row>
@@ -11434,13 +11440,14 @@
       <c r="D6" s="15" t="n">
         <v>16.61</v>
       </c>
-      <c r="E6" s="15" t="n">
+      <c r="E6" s="15"/>
+      <c r="F6" s="15" t="n">
         <v>199.28</v>
       </c>
-      <c r="F6" s="8" t="s">
-        <v>189</v>
-      </c>
       <c r="G6" s="8" t="s">
+        <v>190</v>
+      </c>
+      <c r="H6" s="8" t="s">
         <v>65</v>
       </c>
     </row>
@@ -11457,13 +11464,14 @@
       <c r="D7" s="15" t="n">
         <v>12.78</v>
       </c>
-      <c r="E7" s="15" t="n">
+      <c r="E7" s="15"/>
+      <c r="F7" s="15" t="n">
         <v>153.32</v>
       </c>
-      <c r="F7" s="8" t="s">
-        <v>189</v>
-      </c>
       <c r="G7" s="8" t="s">
+        <v>190</v>
+      </c>
+      <c r="H7" s="8" t="s">
         <v>65</v>
       </c>
     </row>
@@ -11480,13 +11488,14 @@
       <c r="D8" s="15" t="n">
         <v>7.7</v>
       </c>
-      <c r="E8" s="15" t="n">
+      <c r="E8" s="15"/>
+      <c r="F8" s="15" t="n">
         <v>92.35</v>
       </c>
-      <c r="F8" s="8" t="s">
-        <v>189</v>
-      </c>
       <c r="G8" s="8" t="s">
+        <v>190</v>
+      </c>
+      <c r="H8" s="8" t="s">
         <v>65</v>
       </c>
     </row>
@@ -11504,10 +11513,11 @@
       <c r="E9" s="15" t="n">
         <v>9.05</v>
       </c>
-      <c r="F9" s="8" t="s">
-        <v>190</v>
-      </c>
+      <c r="F9" s="15"/>
       <c r="G9" s="8" t="s">
+        <v>191</v>
+      </c>
+      <c r="H9" s="8" t="s">
         <v>65</v>
       </c>
     </row>
@@ -11525,10 +11535,11 @@
       <c r="E10" s="15" t="n">
         <v>9.05</v>
       </c>
-      <c r="F10" s="8" t="s">
-        <v>190</v>
-      </c>
+      <c r="F10" s="15"/>
       <c r="G10" s="8" t="s">
+        <v>191</v>
+      </c>
+      <c r="H10" s="8" t="s">
         <v>65</v>
       </c>
     </row>
@@ -11546,10 +11557,11 @@
       <c r="E11" s="15" t="n">
         <v>7.31</v>
       </c>
-      <c r="F11" s="8" t="s">
-        <v>190</v>
-      </c>
+      <c r="F11" s="15"/>
       <c r="G11" s="8" t="s">
+        <v>191</v>
+      </c>
+      <c r="H11" s="8" t="s">
         <v>65</v>
       </c>
     </row>
@@ -11567,10 +11579,11 @@
       <c r="E12" s="15" t="n">
         <v>18.3</v>
       </c>
-      <c r="F12" s="8" t="s">
-        <v>190</v>
-      </c>
+      <c r="F12" s="15"/>
       <c r="G12" s="8" t="s">
+        <v>191</v>
+      </c>
+      <c r="H12" s="8" t="s">
         <v>65</v>
       </c>
     </row>
@@ -11588,10 +11601,11 @@
       <c r="E13" s="15" t="n">
         <v>18.3</v>
       </c>
-      <c r="F13" s="8" t="s">
-        <v>190</v>
-      </c>
+      <c r="F13" s="15"/>
       <c r="G13" s="8" t="s">
+        <v>191</v>
+      </c>
+      <c r="H13" s="8" t="s">
         <v>65</v>
       </c>
     </row>
@@ -11609,10 +11623,11 @@
       <c r="E14" s="15" t="n">
         <v>12.55</v>
       </c>
-      <c r="F14" s="8" t="s">
-        <v>190</v>
-      </c>
+      <c r="F14" s="15"/>
       <c r="G14" s="8" t="s">
+        <v>191</v>
+      </c>
+      <c r="H14" s="8" t="s">
         <v>65</v>
       </c>
     </row>
@@ -11646,12 +11661,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11662,13 +11677,13 @@
         <v>40</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="F4" s="14" t="s">
         <v>54</v>
@@ -11685,16 +11700,16 @@
         <v>94</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D5" s="15" t="n">
         <v>5</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="G5" s="8" t="s">
         <v>65</v>
@@ -11708,16 +11723,16 @@
         <v>144</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D6" s="15" t="n">
         <v>5</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="G6" s="8" t="s">
         <v>65</v>
@@ -11731,12 +11746,12 @@
         <v>68</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D7" s="15"/>
       <c r="E7" s="8"/>
       <c r="F7" s="8" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="G7" s="8" t="s">
         <v>65</v>
@@ -11774,12 +11789,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11787,28 +11802,28 @@
         <v>39</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H4" s="14" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="I4" s="14" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="J4" s="14" t="s">
         <v>55</v>
@@ -11819,7 +11834,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B5" s="8" t="n">
         <v>10</v>
@@ -11837,16 +11852,16 @@
         <v>62</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="I5" s="8" t="s">
         <v>32</v>
       </c>
       <c r="J5" s="8" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="K5" s="8" t="s">
         <v>65</v>
@@ -11854,7 +11869,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B6" s="8" t="n">
         <v>13</v>
@@ -11872,16 +11887,16 @@
         <v>32</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="I6" s="8" t="s">
         <v>32</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="K6" s="8" t="s">
         <v>65</v>
@@ -11889,7 +11904,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B7" s="8" t="n">
         <v>17</v>
@@ -11907,16 +11922,16 @@
         <v>32</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="I7" s="8" t="s">
         <v>62</v>
       </c>
       <c r="J7" s="8" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="K7" s="8" t="s">
         <v>65</v>
@@ -11924,7 +11939,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B8" s="8" t="n">
         <v>20</v>
@@ -11945,13 +11960,13 @@
         <v>60</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="I8" s="8" t="s">
         <v>32</v>
       </c>
       <c r="J8" s="8" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="K8" s="8" t="s">
         <v>65</v>
@@ -11959,7 +11974,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B9" s="8" t="n">
         <v>25</v>
@@ -11977,16 +11992,16 @@
         <v>32</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="I9" s="8" t="s">
         <v>62</v>
       </c>
       <c r="J9" s="8" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="K9" s="8" t="s">
         <v>65</v>
@@ -11994,7 +12009,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B10" s="8" t="n">
         <v>26</v>
@@ -12015,13 +12030,13 @@
         <v>60</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="I10" s="8" t="s">
         <v>62</v>
       </c>
       <c r="J10" s="8" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="K10" s="8" t="s">
         <v>65</v>
@@ -12029,7 +12044,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B11" s="8" t="n">
         <v>29</v>
@@ -12050,13 +12065,13 @@
         <v>60</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="I11" s="8" t="s">
         <v>62</v>
       </c>
       <c r="J11" s="8" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="K11" s="8" t="s">
         <v>65</v>
@@ -12064,7 +12079,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B12" s="8" t="n">
         <v>37</v>
@@ -12085,13 +12100,13 @@
         <v>60</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="I12" s="8" t="s">
         <v>62</v>
       </c>
       <c r="J12" s="8" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="K12" s="8" t="s">
         <v>65</v>
@@ -12099,7 +12114,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B13" s="8" t="n">
         <v>46</v>
@@ -12117,16 +12132,16 @@
         <v>62</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="I13" s="8" t="s">
         <v>62</v>
       </c>
       <c r="J13" s="8" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="K13" s="8" t="s">
         <v>65</v>
@@ -12134,7 +12149,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B14" s="8" t="n">
         <v>33</v>
@@ -12155,13 +12170,13 @@
         <v>60</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="I14" s="8" t="s">
         <v>62</v>
       </c>
       <c r="J14" s="8" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="K14" s="8" t="s">
         <v>65</v>
@@ -12169,7 +12184,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B15" s="8" t="n">
         <v>27</v>
@@ -12187,16 +12202,16 @@
         <v>62</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="I15" s="8" t="s">
         <v>62</v>
       </c>
       <c r="J15" s="8" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="K15" s="8" t="s">
         <v>65</v>
@@ -12204,7 +12219,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B16" s="8" t="n">
         <v>34</v>
@@ -12225,13 +12240,13 @@
         <v>60</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="I16" s="8" t="s">
         <v>62</v>
       </c>
       <c r="J16" s="8" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="K16" s="8" t="s">
         <v>65</v>
@@ -12239,7 +12254,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B17" s="8" t="n">
         <v>49</v>
@@ -12257,16 +12272,16 @@
         <v>62</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="H17" s="8" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="I17" s="8" t="s">
         <v>62</v>
       </c>
       <c r="J17" s="8" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="K17" s="8" t="s">
         <v>65</v>
@@ -12274,7 +12289,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B18" s="8" t="n">
         <v>41</v>
@@ -12292,16 +12307,16 @@
         <v>32</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="H18" s="8" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="I18" s="8" t="s">
         <v>62</v>
       </c>
       <c r="J18" s="8" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="K18" s="8" t="s">
         <v>65</v>
@@ -12309,7 +12324,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B19" s="8" t="n">
         <v>42</v>
@@ -12327,16 +12342,16 @@
         <v>32</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="H19" s="8" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="I19" s="8" t="s">
         <v>62</v>
       </c>
       <c r="J19" s="8" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="K19" s="8" t="s">
         <v>65</v>
@@ -12344,7 +12359,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B20" s="8" t="n">
         <v>44</v>
@@ -12365,13 +12380,13 @@
         <v>60</v>
       </c>
       <c r="H20" s="8" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="I20" s="8" t="s">
         <v>62</v>
       </c>
       <c r="J20" s="8" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="K20" s="8" t="s">
         <v>65</v>
@@ -12379,7 +12394,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B21" s="8" t="n">
         <v>28</v>
@@ -12397,16 +12412,16 @@
         <v>32</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="H21" s="8" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="I21" s="8" t="s">
         <v>62</v>
       </c>
       <c r="J21" s="8" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="K21" s="8" t="s">
         <v>65</v>
@@ -12414,7 +12429,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B22" s="8" t="n">
         <v>47</v>
@@ -12435,13 +12450,13 @@
         <v>60</v>
       </c>
       <c r="H22" s="8" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="I22" s="8" t="s">
         <v>62</v>
       </c>
       <c r="J22" s="8" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="K22" s="8" t="s">
         <v>65</v>

</xml_diff>

<commit_message>
Rebuild the workbook with the corrected Inputs note
</commit_message>
<xml_diff>
--- a/project-management-pricing-2026-10.xlsx
+++ b/project-management-pricing-2026-10.xlsx
@@ -118,7 +118,7 @@
     <t xml:space="preserve">annual</t>
   </si>
   <si>
-    <t xml:space="preserve">annual or monthly. Annual is cheaper everywhere in this data, by 14% to 37%.</t>
+    <t xml:space="preserve">annual or monthly. Annual is cheaper on all 23 tiers priced both ways, by 7% to 37%.</t>
   </si>
   <si>
     <t xml:space="preserve">WHAT THE TOOL MUST DO</t>
@@ -1875,11 +1875,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="43801790"/>
-        <c:axId val="7178350"/>
+        <c:axId val="93556623"/>
+        <c:axId val="47639396"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="43801790"/>
+        <c:axId val="93556623"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1945,7 +1945,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="7178350"/>
+        <c:crossAx val="47639396"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1953,7 +1953,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="7178350"/>
+        <c:axId val="47639396"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2029,7 +2029,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="43801790"/>
+        <c:crossAx val="93556623"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>